<commit_message>
Fixed time series details calculation + rename of omega parameter
</commit_message>
<xml_diff>
--- a/src/main/resources/downloads/Configuration-sample.xlsx
+++ b/src/main/resources/downloads/Configuration-sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unihk-my.sharepoint.com/personal/najmopa1_uhk_cz/Documents/Bakalářka/GarchApplication/src/main/resources/downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="113" documentId="11_EBD22467C52858873E992CB331CB116ED479E227" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C826354D-B7AE-4696-9976-2C6DBD61B57B}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="11_EBD22467C52858873E992CB331CB116ED479E227" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F695867F-696B-4561-B593-E7C02511E6A3}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,9 +31,6 @@
     <t>Počáteční rozptyl:</t>
   </si>
   <si>
-    <t>Konstantní rozptyl:</t>
-  </si>
-  <si>
     <t>Váhy minulých rozptylů:</t>
   </si>
   <si>
@@ -44,6 +41,9 @@
   </si>
   <si>
     <t>GARCH model sample</t>
+  </si>
+  <si>
+    <t>Konstantní člen:</t>
   </si>
 </sst>
 </file>
@@ -652,10 +652,6 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -976,17 +972,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -996,12 +992,12 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -1011,7 +1007,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1019,17 +1015,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1038,9 +1034,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>0</v>

</xml_diff>

<commit_message>
Rename entities, attributes and classes to match GARCH terminology
</commit_message>
<xml_diff>
--- a/src/main/resources/downloads/Configuration-sample.xlsx
+++ b/src/main/resources/downloads/Configuration-sample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unihk-my.sharepoint.com/personal/najmopa1_uhk_cz/Documents/Bakalářka/GarchApplication/src/main/resources/downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="114" documentId="11_EBD22467C52858873E992CB331CB116ED479E227" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F695867F-696B-4561-B593-E7C02511E6A3}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="11_EBD22467C52858873E992CB331CB116ED479E227" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57AA045E-A15A-4113-921E-A1FE9C252128}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,12 +31,6 @@
     <t>Počáteční rozptyl:</t>
   </si>
   <si>
-    <t>Váhy minulých rozptylů:</t>
-  </si>
-  <si>
-    <t>Váhy minulých odhadů:</t>
-  </si>
-  <si>
     <t>Configuration sample</t>
   </si>
   <si>
@@ -44,6 +38,12 @@
   </si>
   <si>
     <t>Konstantní člen:</t>
+  </si>
+  <si>
+    <t>Alfa koeficienty:</t>
+  </si>
+  <si>
+    <t>Beta koeficienty:</t>
   </si>
 </sst>
 </file>
@@ -623,11 +623,27 @@
           </a:r>
           <a:r>
             <a:rPr lang="cs-CZ" sz="1100" baseline="0"/>
-            <a:t> minulých rozptylů </a:t>
+            <a:t> předchozích reziduí </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="el-GR"/>
-            <a:t>(β)</a:t>
+            <a:t>(</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>α</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR"/>
+            <a:t>)</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="cs-CZ" sz="1100" baseline="0"/>
@@ -635,7 +651,23 @@
           </a:r>
           <a:r>
             <a:rPr lang="el-GR"/>
-            <a:t>(α)</a:t>
+            <a:t>(</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>β</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="el-GR"/>
+            <a:t>)</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="cs-CZ"/>
@@ -652,6 +684,10 @@
     <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -972,17 +1008,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -992,12 +1028,12 @@
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -1007,7 +1043,7 @@
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1015,17 +1051,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1034,9 +1070,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B6">
         <v>0</v>

</xml_diff>